<commit_message>
edim-ai-blueprint: i18n 확정 — KO 기본 + EN/JA/ZH 전 문서 관통
- REQ-N-015 확정(4로케일 100%·KO 폴백) · 기능 SYS-021 신설(179) · 메뉴 98(다국어 관리)
- DB v0.5: sys_translation 신설(54테이블) — 미결정 #7 해소(컬럼 방식 기각, 번역 테이블 채택),
  locale 공통코드, DDL 반영 + 실 PG 적용·CJK 저장 스모크(en/ja/zh) 통과
- API 108: GET /i18n/{locale}·PUT /i18n/translations, Accept-Language 헤더 규약
- 개발표준 §4 i18n 절: 리소스 키·locale 우선순위·Intl 포맷·CJK 폰트 스택·EN+30% 확장
- 연쇄 재생성: 요구사항→기능→메뉴→권한→RTM(179/179)→FVT(179+22)→OpenAPI(107op 검증)
</commit_message>
<xml_diff>
--- a/edim-ai-blueprint/docs/02_요구사항/EDIM_요구사항정의서.xlsx
+++ b/edim-ai-blueprint/docs/02_요구사항/EDIM_요구사항정의서.xlsx
@@ -1454,7 +1454,7 @@
       </c>
       <c r="H7" s="22" t="inlineStr">
         <is>
-          <t>SYS-013~020</t>
+          <t>SYS-013~021</t>
         </is>
       </c>
       <c r="I7" s="22" t="inlineStr"/>
@@ -3842,20 +3842,24 @@
       </c>
       <c r="D16" s="22" t="inlineStr">
         <is>
-          <t>다국어</t>
+          <t>다국어 (i18n)</t>
         </is>
       </c>
       <c r="E16" s="22" t="inlineStr">
         <is>
-          <t>한국어 기본, 다국어 확장 구조(i18n)</t>
+          <t>한국어 기본 + 영어·일본어·중국어 지원 — UI 리소스 번들 + 데이터 라벨 번역(sys_translation), 로케일별 날짜·숫자·통화 포맷, 번역 누락 시 KO 폴백</t>
         </is>
       </c>
       <c r="F16" s="22" t="inlineStr">
         <is>
-          <t>영어 1차 (협의)</t>
-        </is>
-      </c>
-      <c r="G16" s="22" t="inlineStr"/>
+          <t>4개 로케일(ko/en/ja/zh) 전환 100%</t>
+        </is>
+      </c>
+      <c r="G16" s="22" t="inlineStr">
+        <is>
+          <t>확정 (2026-07-07)</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="n">

</xml_diff>